<commit_message>
Logos FEN/FCFM/DII, programa interfacultades, PDF completo por tesis, boton de descarga
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YRc6gMzAmr2dLwJ4q8rmXs
</commit_message>
<xml_diff>
--- a/catalogo_tesis_MAN.xlsx
+++ b/catalogo_tesis_MAN.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM15"/>
+  <dimension ref="A1:AN15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,7 @@
     <col width="45" customWidth="1" min="37" max="37"/>
     <col width="40" customWidth="1" min="38" max="38"/>
     <col width="40" customWidth="1" min="39" max="39"/>
+    <col width="40" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -668,6 +669,11 @@
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
+          <t>PDF en el sitio</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
           <t>Notas</t>
         </is>
       </c>
@@ -848,6 +854,11 @@
       </c>
       <c r="AL2" s="2" t="inlineStr"/>
       <c r="AM2" s="2" t="inlineStr">
+        <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-quintanilla.pdf</t>
+        </is>
+      </c>
+      <c r="AN2" s="2" t="inlineStr">
         <is>
           <t>El texto incluye resumen ejecutivo y abstract. Las tablas aparecen al final del archivo, separadas de sus títulos en el cuerpo. No se nombra una contraparte institucional formal: se usan fuentes públicas de ChileCompra sin convenio con una organización. El modelo 'es-specific' se menciona sin nombre completo. Los LLMs con prompts se mencionan solo como trabajo futuro, no se aplican.</t>
         </is>
@@ -1030,6 +1041,11 @@
       <c r="AL3" s="2" t="inlineStr"/>
       <c r="AM3" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-celedon.pdf</t>
+        </is>
+      </c>
+      <c r="AN3" s="2" t="inlineStr">
+        <is>
           <t>La tesis aplica además AR, MA, ARMA, ARIMA, Random Forest, HistGradientBoosting, Elastic Net, Naive Seasonal, Diebold-Mariano con Newey-West y Holm, Model Confidence Set con bootstrap estacionario y pruebas ADF, KPSS y Ljung-Box; se omitieron de techniques por el límite de 10. La organización no se nombra en el texto. El texto incluye dedicatoria y agradecimientos extensos con nombres personales.</t>
         </is>
       </c>
@@ -1207,6 +1223,11 @@
       <c r="AL4" s="2" t="inlineStr"/>
       <c r="AM4" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-cabezas.pdf</t>
+        </is>
+      </c>
+      <c r="AN4" s="2" t="inlineStr">
+        <is>
           <t>El texto extraído comienza en el capítulo de metodología: no incluye portada, resumen, introducción ni marco teórico. Hay inconsistencia en el período de datos (1998-2023 en la descripción del enfoque, 1960-2023 en resultados). Las tablas y gráficos no están en el texto, por lo que no se dispone de RMSE ni de métricas de Random Forest en prueba.</t>
         </is>
       </c>
@@ -1388,6 +1409,11 @@
       <c r="AL5" s="2" t="inlineStr"/>
       <c r="AM5" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-torres.pdf</t>
+        </is>
+      </c>
+      <c r="AN5" s="2" t="inlineStr">
+        <is>
           <t>Las secciones referidas en la discusión (8.2.5, 8.2.6, 8.3.2) no coinciden con la numeración del informe. Hay inconsistencias menores en cifras entre secciones: el coeficiente de pct_diputados aparece como +0,2037 en la tabla OLS y +0,279 en conclusiones; la importancia de XGBoost se cita como 0,45 en conclusiones pero 0,188 por gain en la tabla. Año en portada: 2026.</t>
         </is>
       </c>
@@ -1569,6 +1595,11 @@
       <c r="AL6" s="2" t="inlineStr"/>
       <c r="AM6" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-gutierrez.pdf</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
           <t>Trabajo orientado a los Servicios de Salud Reloncaví, Chiloé y Osorno como contraparte institucional, pero los datos usados son públicos (DEIS) y no se declara convenio formal, por lo que organization se deja en null. La valorización económica (396 a 793 millones de pesos anuales) es un ejercicio ilustrativo, no un resultado del modelo. Fecha de la portada: junio 2026; profesor guía Richard Weber.</t>
         </is>
       </c>
@@ -1750,6 +1781,11 @@
       <c r="AL7" s="2" t="inlineStr"/>
       <c r="AM7" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-delrio.pdf</t>
+        </is>
+      </c>
+      <c r="AN7" s="2" t="inlineStr">
+        <is>
           <t>Tesis fechada 2026 (Actividad Formativa Equivalente), profesor guía Charles Thraves. Las predicciones sobre 2025 son retrospectivas: el resultado ya era conocido y la asignación manual de ese ciclo se ajustó al resultado observado (sesgo retrospectivo declarado por el autor). El modelo Beta=0 no alcanza optimalidad certificada en CBC y no es replicable entre corridas. Los anexos del texto solo contienen nombres de figuras, sin contenido.</t>
         </is>
       </c>
@@ -1931,6 +1967,11 @@
       <c r="AL8" s="2" t="inlineStr"/>
       <c r="AM8" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2026-hernandez.pdf</t>
+        </is>
+      </c>
+      <c r="AN8" s="2" t="inlineStr">
+        <is>
           <t>La portada indica 'Borrador Final' (abril 2026). Es una tesis de ingeniería de datos geoespaciales y producto (plataformas Catastral.cl y combustible.tremen.tech), no de modelamiento predictivo: no se entrenan modelos de ML; CLIP se usa como clasificador satelital preentrenado en el caso aplicado. El texto menciona Newmark Chile 'en el Capítulo 1' pero ese contexto no aparece en el documento. Algunas referencias cruzadas de sección son inconsistentes (p.ej. 'Sección 4.2.2' por 7.4.2).</t>
         </is>
       </c>
@@ -2115,6 +2156,11 @@
         </is>
       </c>
       <c r="AM9" s="2" t="inlineStr">
+        <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-canete.pdf</t>
+        </is>
+      </c>
+      <c r="AN9" s="2" t="inlineStr">
         <is>
           <t>La empresa no se nombra, aunque las gerencias listadas en el anexo (Transporte de Pasajeros, Extensiones, Obras Civiles) y la categoría de sindicato S_Metro sugieren un operador de transporte urbano. El texto no menciona lenguaje ni librerías. Hay una inconsistencia de signo: la metodología define persuasibles con uplift positivo, pero en los resultados los persuasibles son los de uplift score menor a -0,05 (moda en -1,0), ya que el outcome es la renuncia. La tabla 4 y el gráfico 8 están en anexos; los gráficos no se recuperan en el texto extraído.</t>
         </is>
@@ -2297,6 +2343,11 @@
       </c>
       <c r="AM10" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-araneda.pdf</t>
+        </is>
+      </c>
+      <c r="AN10" s="2" t="inlineStr">
+        <is>
           <t>El texto extraído no incluye las tablas en su lugar original: aparecen al final en formato de columnas separadas por barras verticales. El lenguaje Python no se menciona de forma explícita; se infiere por las librerías citadas (scikit-learn, transformers de Hugging Face, pysentimiento). Se evaluaron además BETO (nlptown), TextBlob y VADER como modelos de sentimiento, descartados por menor desempeño. Fecha de la portada: junio 2025.</t>
         </is>
       </c>
@@ -2482,6 +2533,11 @@
       </c>
       <c r="AM11" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-barros.pdf</t>
+        </is>
+      </c>
+      <c r="AN11" s="2" t="inlineStr">
+        <is>
           <t>La portada del texto extraído dice 'Determinación de las variables que explican eficiencia en establecimientos educacionales de Chile' (2025, profesora guía Felix Lizama); se usó el título oficial entregado. El resumen ejecutivo es más bien una declaración de objetivos; las cifras provienen de los capítulos de resultados y anexos. El tamaño de la muestra (912) se infiere de la tabla descriptiva del anexo 5 (valores únicos de DMU), no se declara explícitamente. Hay inconsistencias internas sobre el signo del efecto de la razón de horas de aula por alumno: el cuerpo y el anexo 10 lo describen como inverso, mientras el análisis por cuartiles y el anexo 9 lo describen como positivo. Las métricas se denominan 'de clasificación' aunque el problema es de regresión. Más de la mitad del texto son anexos con descripciones de gráficos SHAP.</t>
         </is>
       </c>
@@ -2667,6 +2723,11 @@
       </c>
       <c r="AM12" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-sepulveda.pdf</t>
+        </is>
+      </c>
+      <c r="AN12" s="2" t="inlineStr">
+        <is>
           <t>El texto tiene inconsistencias internas: la síntesis de P4 reporta 720 reclamos de seguridad alimentaria con 45/32/23 % de estrategias y notas 3,4/2,7/2,1, mientras que la sección correspondiente reporta 72 casos, 26,1 % evasivas, 73,9 % técnicas y cero transparentes (se usó esta última versión en los highlights). La base completa aparece como 5.465 y también como 5.468 evaluaciones. Hay párrafos duplicados en la sección de seguridad alimentaria y dos secciones tituladas Conclusiones. El OE5 se cita en la metodología pero no está en la lista de objetivos. No se nombra explícitamente el lenguaje de programación; el anexo muestra prompts en sintaxis tipo Python (SYSTEM_CONTENT = """..."""). Declara uso de Claude, ChatGPT y Gemini para mejorar la redacción.</t>
         </is>
       </c>
@@ -2852,6 +2913,11 @@
       </c>
       <c r="AM13" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-gajardo.pdf</t>
+        </is>
+      </c>
+      <c r="AN13" s="2" t="inlineStr">
+        <is>
           <t>El texto no nombra explícitamente el lenguaje; se infiere Python por las referencias a MinMaxScaler, seasonal_decompose, DataFrame, Adam y EarlyStopping. Se menciona que el modelo se orienta a un portfolio manager de un banco de inversión, pero no se identifica ninguna organización. Las tablas de machine learning (5 a 10) reportan RMSE pero el texto las llama repetidamente 'rentabilidad', lo que genera confusión; el resumen ejecutivo repite ese uso. Hay dos tablas numeradas como Tabla 2 y los gráficos ARIMA/SARIMAX y los boxplots del anexo no se extrajeron del PDF.</t>
         </is>
       </c>
@@ -3037,6 +3103,11 @@
       </c>
       <c r="AM14" s="2" t="inlineStr">
         <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-ceroni.pdf</t>
+        </is>
+      </c>
+      <c r="AN14" s="2" t="inlineStr">
+        <is>
           <t>Documento rotulado como Taller AFE, Informe 3 (AFE para optar al grado), profesor guía Richard Weber, 2025. Resumen ejecutivo en español e inglés incluido. Las tablas y gráficos aparecen como texto al final. Inconsistencia menor: el texto dice que todos los R cuadrado por estilo superan 0,82, pero la tabla muestra Witbier con 0,77. Los modelos de clasificación (KNN, Random Forest, redes neuronales, SVM) se probaron como análisis alternativo y se descartaron.</t>
         </is>
       </c>
@@ -3225,6 +3296,11 @@
         </is>
       </c>
       <c r="AM15" s="2" t="inlineStr">
+        <is>
+          <t>https://man-thesis-catalog.vercel.app/pdf/2025-yanez.pdf</t>
+        </is>
+      </c>
+      <c r="AN15" s="2" t="inlineStr">
         <is>
           <t>Informe final fechado en enero de 2025. El texto extraído perdió las ecuaciones y los contenidos de varias figuras y tablas; algunas tablas de resultados (A/E mensuales 2024) solo aparecen como títulos. Se detecta una inconsistencia menor: el MSE 824,35 se reporta para GRU y luego se atribuye a LSTM y GRU en conjunto. El autor no entrega el MSE numérico del LSTM de serie temporal.</t>
         </is>
@@ -4345,12 +4421,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial, Universidad de Chile</t>
+          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering, Universidad de Chile</t>
+          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4383,12 +4459,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Administración, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Administración, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Department of Management, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4421,12 +4497,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Administración, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Administración, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Department of Management, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -4459,12 +4535,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Control de Gestión y Sistemas de Información, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Control de Gestión y Sistemas de Información, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Department of Management Control and Information Systems, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management Control and Information Systems, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -4497,12 +4573,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial, Universidad de Chile</t>
+          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering, Universidad de Chile</t>
+          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4535,12 +4611,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial, Universidad de Chile</t>
+          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering, Universidad de Chile</t>
+          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -4611,12 +4687,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Administración, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Administración, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Department of Management, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -4649,12 +4725,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>School of Economics and Business, Universidad de Chile</t>
+          <t>School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -4687,12 +4763,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial, Universidad de Chile</t>
+          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering, Universidad de Chile</t>
+          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -4725,12 +4801,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Administración, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Administración, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Department of Management, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -4801,12 +4877,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Control de Gestión y Sistemas de Información, Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Departamento de Control de Gestión y Sistemas de Información, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Department of Management Control and Information Systems, School of Economics and Business, Universidad de Chile</t>
+          <t>Department of Management Control and Information Systems, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -4839,12 +4915,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial, Universidad de Chile</t>
+          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering, Universidad de Chile</t>
+          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -4877,12 +4953,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Facultad de Economía y Negocios, Universidad de Chile</t>
+          <t>Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>School of Economics and Business, Universidad de Chile</t>
+          <t>School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Filtros sin saltos de scroll, Olivares en FEN, links de Maldonado y Vergara
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YRc6gMzAmr2dLwJ4q8rmXs
</commit_message>
<xml_diff>
--- a/catalogo_tesis_MAN.xlsx
+++ b/catalogo_tesis_MAN.xlsx
@@ -4765,7 +4765,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://fen.uchile.cl/es/academicos-investigacion/directorio-de-academicos/detalle/sebastian-maldonado</t>
+          <t>https://fen.uchile.cl/es/academicos-investigacion/directorio-de-academicos/detalle/sebastian-maldonado-3</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4831,17 +4831,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Departamento de Ingeniería Industrial (DII), Facultad de Ciencias Físicas y Matemáticas (FCFM), Universidad de Chile</t>
+          <t>Departamento de Administración, Facultad de Economía y Negocios (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Department of Industrial Engineering (DII), School of Physical and Mathematical Sciences (FCFM), Universidad de Chile</t>
+          <t>Department of Management, School of Economics and Business (FEN), Universidad de Chile</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.dii.uchile.cl/quien/marcelo-olivares/</t>
+          <t>https://fen.uchile.cl/es/academicos-investigacion/directorio-de-academicos/detalle/marcelo-olivares</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4879,12 +4879,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.researchgate.net/profile/Cinthya-Vergara-Silva</t>
+          <t>https://www.linkedin.com/in/cinthya-leonor-vergara-silva-6298b221/</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>personal</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">

</xml_diff>